<commit_message>
refactor: centralize app paths and resources
</commit_message>
<xml_diff>
--- a/data/yearly_template.xlsx
+++ b/data/yearly_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -137,9 +137,6 @@
   </si>
   <si>
     <t xml:space="preserve">May</t>
-  </si>
-  <si>
-    <t xml:space="preserve">d</t>
   </si>
   <si>
     <t xml:space="preserve">Jun</t>
@@ -597,7 +594,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:U34"/>
+  <dimension ref="A1:T34"/>
   <sheetFormatPr defaultColWidth="7.66015625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="257" min="1" style="1" width="7.66"/>
@@ -617,13 +614,13 @@
       <c r="F1" s="5"/>
       <c r="G1" s="4"/>
       <c r="H1" s="4"/>
-      <c r="I1" s="0"/>
-      <c r="J1" s="0"/>
+      <c r="I1" s="6"/>
+      <c r="J1" s="6"/>
       <c r="K1" s="4"/>
       <c r="L1" s="4"/>
       <c r="M1" s="4"/>
-      <c r="N1" s="0"/>
-      <c r="O1" s="0"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
       <c r="P1" s="6"/>
       <c r="Q1" s="7"/>
       <c r="R1" s="7"/>
@@ -647,7 +644,7 @@
         <v>4</v>
       </c>
       <c r="J2" s="5"/>
-      <c r="K2" s="0"/>
+      <c r="K2" s="6"/>
       <c r="L2" s="4"/>
       <c r="M2" s="4"/>
       <c r="N2" s="5" t="s">
@@ -679,7 +676,7 @@
       <c r="J3" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="0"/>
+      <c r="K3" s="6"/>
       <c r="L3" s="6"/>
       <c r="M3" s="7"/>
       <c r="N3" s="5" t="s">
@@ -709,7 +706,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="9"/>
-      <c r="K4" s="0"/>
+      <c r="K4" s="6"/>
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
       <c r="N4" s="5" t="s">
@@ -925,16 +922,13 @@
       <c r="R11" s="24"/>
       <c r="S11" s="24"/>
       <c r="T11" s="17"/>
-      <c r="U11" s="1" t="s">
-        <v>39</v>
-      </c>
     </row>
     <row r="12" customFormat="false" ht="16.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="18" t="n">
         <v>3</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C12" s="23"/>
       <c r="D12" s="24"/>
@@ -960,7 +954,7 @@
         <v>4</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C13" s="23"/>
       <c r="D13" s="24"/>
@@ -986,7 +980,7 @@
         <v>5</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C14" s="23"/>
       <c r="D14" s="24"/>
@@ -1012,7 +1006,7 @@
         <v>6</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C15" s="23"/>
       <c r="D15" s="24"/>
@@ -1038,7 +1032,7 @@
         <v>7</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C16" s="23"/>
       <c r="D16" s="24"/>
@@ -1064,7 +1058,7 @@
         <v>8</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C17" s="23"/>
       <c r="D17" s="24"/>
@@ -1090,7 +1084,7 @@
         <v>9</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C18" s="23"/>
       <c r="D18" s="24"/>
@@ -1116,7 +1110,7 @@
         <v>10</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C19" s="23"/>
       <c r="D19" s="24"/>
@@ -1142,7 +1136,7 @@
         <v>11</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C20" s="23"/>
       <c r="D20" s="24"/>
@@ -1168,7 +1162,7 @@
         <v>12</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C21" s="23"/>
       <c r="D21" s="24"/>
@@ -1194,7 +1188,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C22" s="26"/>
       <c r="D22" s="26"/>
@@ -1280,17 +1274,17 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="27" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" s="29" t="s">
         <v>51</v>
-      </c>
-      <c r="C26" s="29" t="s">
-        <v>52</v>
       </c>
       <c r="D26" s="29"/>
       <c r="E26" s="30"/>
       <c r="F26" s="30"/>
       <c r="G26" s="30"/>
       <c r="H26" s="29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I26" s="29"/>
       <c r="J26" s="29"/>
@@ -1299,7 +1293,7 @@
       <c r="M26" s="29"/>
       <c r="N26" s="29"/>
       <c r="O26" s="29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1471,9 +1465,7 @@
       <c r="S34" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="E1:F1"/>
-    <mergeCell ref="N2:O2"/>
+  <mergeCells count="7">
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="N4:O4"/>
     <mergeCell ref="A6:S6"/>

</xml_diff>

<commit_message>
fix: improve empty and error states
</commit_message>
<xml_diff>
--- a/data/yearly_template.xlsx
+++ b/data/yearly_template.xlsx
@@ -1475,11 +1475,11 @@
     <mergeCell ref="J8:S8"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.236111111111111" right="0.236111111111111" top="0.501388888888889" bottom="0.501388888888889" header="0.236111111111111" footer="0.236111111111111"/>
+  <pageMargins left="0.236111111111111" right="0.236111111111111" top="0.334722222222222" bottom="0.334722222222222" header="0.236111111111111" footer="0.236111111111111"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" firstPageNumber="1" useFirstPageNumber="true" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader>&amp;C&amp;"Times New Roman"&amp;12&amp;A</oddHeader>
-    <oddFooter>&amp;C&amp;"Times New Roman"&amp;12Page &amp;P</oddFooter>
+    <oddHeader/>
+    <oddFooter/>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>